<commit_message>
correcciones Reglas - y recuperacion de la cagada del merge :( jsjs
</commit_message>
<xml_diff>
--- a/usuarios.xlsx
+++ b/usuarios.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3BE033D-B6FC-4E60-AE47-6866CAAAA26C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F070CDF-6C63-42DE-8424-84249E45D353}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="30">
   <si>
     <t>ID / Cédula</t>
   </si>
@@ -99,6 +99,12 @@
   </si>
   <si>
     <t>RRH</t>
+  </si>
+  <si>
+    <t>OSCAR</t>
+  </si>
+  <si>
+    <t>COVA</t>
   </si>
 </sst>
 </file>
@@ -153,13 +159,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -499,7 +504,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.5703125" customWidth="1"/>
@@ -508,7 +513,7 @@
     <col min="4" max="4" width="20.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -522,7 +527,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>16335012</v>
       </c>
@@ -536,7 +541,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>24765865</v>
       </c>
@@ -550,7 +555,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>26082578</v>
       </c>
@@ -564,7 +569,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>17654625</v>
       </c>
@@ -578,7 +583,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>31993594</v>
       </c>
@@ -593,7 +598,7 @@
       </c>
       <c r="F6" s="2"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>29591045</v>
       </c>
@@ -607,7 +612,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>11111111</v>
       </c>
@@ -621,8 +626,8 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9">
         <v>2</v>
       </c>
       <c r="B9" t="s">
@@ -635,8 +640,8 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10">
         <v>22652518</v>
       </c>
       <c r="B10" t="s">
@@ -649,8 +654,16 @@
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="H12" s="3"/>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>11143945</v>
+      </c>
+      <c r="B11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" t="s">
+        <v>29</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>